<commit_message>
Actualiza gitignore y agrega estructura del proyecto
</commit_message>
<xml_diff>
--- a/salida/facturas_extraidas.xlsx
+++ b/salida/facturas_extraidas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -580,37 +580,37 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1790556677001</t>
+          <t>1790112233001</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Banco Productivo Nacional</t>
+          <t>Banco Meridiano</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>001-099-000456789</t>
+          <t>001-003-000078451</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>18/03/2025</t>
+          <t>22/06/2025</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>1803202501179055667700120010990004567890045678912</t>
+          <t>2206202501179011223300120010030000784510007845112</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Comisión por servicios bancarios - mantenimiento de cuenta y transferencias</t>
+          <t>Comisión por servicios de custodia de valores</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>1.850,00</t>
+          <t>610,00</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -620,17 +620,17 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>277,50</t>
+          <t>91,50</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2.127,50</t>
+          <t>701,50</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>banco_productivo_nacional</t>
+          <t>ia_gemini</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -643,37 +643,37 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1791223344001</t>
+          <t>1790556677001</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Banco Solidaridad Andina</t>
+          <t>Banco Productivo Nacional</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>001-002-000000451</t>
+          <t>001-099-000456789</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>15/01/2025</t>
+          <t>18/03/2025</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1202501151791223344001120010020000004510012001099</t>
+          <t>1803202501179055667700120010990004567890045678912</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>COMISION MANTENIMIENTO DE CUENTA</t>
+          <t>Comisión por servicios bancarios - mantenimiento de cuenta y transferencias</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>52.50</t>
+          <t>1.850,00</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -683,17 +683,17 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>7.88</t>
+          <t>277,50</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>60.38</t>
+          <t>2.127,50</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>banco_solidaridad_andina</t>
+          <t>banco_productivo_nacional</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -716,17 +716,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>001-002-000000487</t>
+          <t>001-002-000000451</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>14/02/2025</t>
+          <t>15/01/2025</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>1202502141791223344001120010020000004870012001099</t>
+          <t>1202501151791223344001120010020000004510012001099</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>55.40</t>
+          <t>52.50</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -746,12 +746,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>8.31</t>
+          <t>7.88</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>63.71</t>
+          <t>60.38</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -779,17 +779,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>001-002-000000523</t>
+          <t>001-002-000000487</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>17/03/2025</t>
+          <t>14/02/2025</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1202503171791223344001120010020000005230012001099</t>
+          <t>1202502141791223344001120010020000004870012001099</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>60.50</t>
+          <t>55.40</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -809,12 +809,12 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>9.07</t>
+          <t>8.31</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>69.57</t>
+          <t>63.71</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -842,17 +842,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>001-002-000000559</t>
+          <t>001-002-000000523</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>17/03/2025</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1202504161791223344001120010020000005590012001099</t>
+          <t>1202503171791223344001120010020000005230012001099</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>57.00</t>
+          <t>60.50</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -872,12 +872,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>8.55</t>
+          <t>9.07</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>65.55</t>
+          <t>69.57</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -905,17 +905,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>001-002-000000594</t>
+          <t>001-002-000000559</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>15/05/2025</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1202505151791223344001120010020000005940012001099</t>
+          <t>1202504161791223344001120010020000005590012001099</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>60.25</t>
+          <t>57.00</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>9.04</t>
+          <t>8.55</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>69.29</t>
+          <t>65.55</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -958,37 +958,37 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>1790998877001</t>
+          <t>1791223344001</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Tarjeta Cumbre Elite Pay</t>
+          <t>Banco Solidaridad Andina</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>001-003-000054321</t>
+          <t>001-002-000000594</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>18/03/2025</t>
+          <t>15/05/2025</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>1803202501179099887700120030005432100054321301</t>
+          <t>1202505151791223344001120010020000005940012001099</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>COMISION MANTENIMIENTO TARJETA ELITE PAY</t>
+          <t>COMISION MANTENIMIENTO DE CUENTA</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>22.40</t>
+          <t>60.25</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -998,17 +998,17 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>9.04</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>25.76</t>
+          <t>69.29</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>tarjeta_cumbre_elite_pay</t>
+          <t>banco_solidaridad_andina</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1021,17 +1021,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>1790667788001</t>
+          <t>1790998877001</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Tarjeta Cumbre Nortis</t>
+          <t>Tarjeta Cumbre Elite Pay</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>001-002-000098765</t>
+          <t>001-003-000054321</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1041,17 +1041,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>1803202501179066778800120020009876500098765201</t>
+          <t>1803202501179099887700120030005432100054321301</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>COMISION MANTENIMIENTO TARJETA NORTIS</t>
+          <t>COMISION MANTENIMIENTO TARJETA ELITE PAY</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>13.45</t>
+          <t>22.40</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1061,17 +1061,17 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>15.47</t>
+          <t>25.76</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>tarjeta_cumbre_nortis</t>
+          <t>tarjeta_cumbre_elite_pay</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1084,17 +1084,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>1790334455001</t>
+          <t>1790667788001</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Tarjeta Cumbre Prisma</t>
+          <t>Tarjeta Cumbre Nortis</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>001-004-000112567</t>
+          <t>001-002-000098765</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1104,17 +1104,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>1803202501179033445500120010040001125670011256701</t>
+          <t>1803202501179066778800120020009876500098765201</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>COMISION MANTENIMIENTO TARJETA PRISMA</t>
+          <t>COMISION MANTENIMIENTO TARJETA NORTIS</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>18.90</t>
+          <t>13.45</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1124,17 +1124,17 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2.84</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>21.74</t>
+          <t>15.47</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>tarjeta_cumbre_prisma</t>
+          <t>tarjeta_cumbre_nortis</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1152,60 +1152,123 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>Tarjeta Cumbre Prisma</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>001-004-000112567</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>18/03/2025</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>1803202501179033445500120010040001125670011256701</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>COMISION MANTENIMIENTO TARJETA PRISMA</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>18.90</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>2.84</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>21.74</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>tarjeta_cumbre_prisma</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>válida</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1790334455001</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
           <t>Tarjeta Cumbre Zenith</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>001-004-000112233</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>18/03/2025</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>1803202501179033445500120010040001122330011223301</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>COMISION MANTENIMIENTO TARJETA ZENITH</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>15.50</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>2.33</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>17.83</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>tarjeta_cumbre_zenith</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>válida</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>